<commit_message>
20250702 - update of included studies table
</commit_message>
<xml_diff>
--- a/data_u1/included_studies_2025-01-16_LSR3_H.xlsx
+++ b/data_u1/included_studies_2025-01-16_LSR3_H.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sksiafis/Desktop/LSR3_taar1_H_2025.01.16/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sksiafis/Documents/GitHub/LSR3_taar1_H/data_u1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3429374-089F-304A-89EF-D0FFBAE26EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC32EA9-3CAB-AB44-9EE4-278133C65F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23000" yWindow="-21600" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5300" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of included studies" sheetId="9" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="314">
   <si>
     <t>ID</t>
   </si>
@@ -877,9 +877,6 @@
     <t>F-DOPA PET</t>
   </si>
   <si>
-    <t>August 7, 2019</t>
-  </si>
-  <si>
     <t>June 6, 2023</t>
   </si>
   <si>
@@ -935,6 +932,54 @@
   </si>
   <si>
     <t>November 9 2023</t>
+  </si>
+  <si>
+    <t>August 7 2019</t>
+  </si>
+  <si>
+    <t>NCT06880328 (2019)</t>
+  </si>
+  <si>
+    <t>NCT06894212 (2025)</t>
+  </si>
+  <si>
+    <t>18F-Dihydroxyphenylalanine (DOPA) Positron Emission Tomography (PET) Study to Explore Dopamine Synthesis Capacity in the Whole Striatum After 2 Weeks of Treatment With Ralmitaront or Placebo in Participants With Schizophrenia</t>
+  </si>
+  <si>
+    <t>A Trial of the Efficacy and Safety of SEP-363856 in Acutely Psychotic Participants With Schizophrenia</t>
+  </si>
+  <si>
+    <t>BP39833</t>
+  </si>
+  <si>
+    <t>DB-RCT two-period crossover; 2 weeks (phase 1)</t>
+  </si>
+  <si>
+    <t>382-201-00035</t>
+  </si>
+  <si>
+    <t>Otsuka</t>
+  </si>
+  <si>
+    <t>Ralmitaront 150 mg/d; Placebo</t>
+  </si>
+  <si>
+    <t>Ulotaront 75mg; Ulotaront 100mg; Placebo</t>
+  </si>
+  <si>
+    <t>F-DOPA PET; fMRI; tolerability</t>
+  </si>
+  <si>
+    <t>November 07 2018</t>
+  </si>
+  <si>
+    <t>September 04 2019</t>
+  </si>
+  <si>
+    <t>February 25 2025</t>
+  </si>
+  <si>
+    <t>August 31 2028</t>
   </si>
 </sst>
 </file>
@@ -1394,7 +1439,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE07FD7C-2BB8-4877-BC1B-2964FB11D2BE}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="27" customWidth="1"/>
@@ -1518,7 +1563,7 @@
         <v>74</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H3" s="9">
         <v>131</v>
@@ -1536,7 +1581,7 @@
         <v>2023</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="N3" s="9" t="s">
         <v>77</v>
@@ -1750,7 +1795,7 @@
         <v>246</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="L8" t="s">
         <v>86</v>
@@ -1926,13 +1971,13 @@
         <v>249</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="L12" s="9">
         <v>2023</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="N12" t="s">
         <v>72</v>
@@ -2111,7 +2156,7 @@
         <v>2</v>
       </c>
       <c r="N16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2366,7 +2411,7 @@
         <v>260</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="L22" s="14">
         <v>2024</v>
@@ -2392,10 +2437,10 @@
         <v>88</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>211</v>
@@ -2410,7 +2455,7 @@
         <v>261</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="L23" s="14">
         <v>2024</v>
@@ -2483,10 +2528,10 @@
         <v>212</v>
       </c>
       <c r="F25" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="G25" s="12" t="s">
         <v>285</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>286</v>
       </c>
       <c r="H25" s="11">
         <v>31</v>
@@ -2498,7 +2543,7 @@
         <v>262</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="L25" s="9">
         <v>2023</v>
@@ -2507,7 +2552,7 @@
         <v>2</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2800,19 +2845,19 @@
         <v>463</v>
       </c>
       <c r="I32" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J32" t="s">
         <v>150</v>
       </c>
       <c r="K32" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="L32" s="14">
         <v>2023</v>
       </c>
       <c r="M32" s="14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="N32" t="s">
         <v>72</v>
@@ -2888,13 +2933,13 @@
         <v>101</v>
       </c>
       <c r="I34" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J34" t="s">
         <v>153</v>
       </c>
       <c r="K34" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="L34" s="14">
         <v>2024</v>
@@ -2932,7 +2977,7 @@
         <v>67</v>
       </c>
       <c r="I35" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J35" t="s">
         <v>156</v>
@@ -2979,10 +3024,10 @@
         <v>278</v>
       </c>
       <c r="J36" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="K36" s="2" t="s">
         <v>279</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="L36">
         <v>2023</v>
@@ -2991,7 +3036,92 @@
         <v>2</v>
       </c>
       <c r="N36" t="s">
-        <v>281</v>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>299</v>
+      </c>
+      <c r="B37" t="s">
+        <v>301</v>
+      </c>
+      <c r="C37" t="s">
+        <v>303</v>
+      </c>
+      <c r="D37" t="s">
+        <v>69</v>
+      </c>
+      <c r="E37" t="s">
+        <v>304</v>
+      </c>
+      <c r="F37" t="s">
+        <v>99</v>
+      </c>
+      <c r="G37" t="s">
+        <v>307</v>
+      </c>
+      <c r="H37">
+        <v>35</v>
+      </c>
+      <c r="I37" t="s">
+        <v>309</v>
+      </c>
+      <c r="J37" t="s">
+        <v>310</v>
+      </c>
+      <c r="K37" t="s">
+        <v>311</v>
+      </c>
+      <c r="L37">
+        <v>2019</v>
+      </c>
+      <c r="M37" t="s">
+        <v>2</v>
+      </c>
+      <c r="N37" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>300</v>
+      </c>
+      <c r="B38" t="s">
+        <v>302</v>
+      </c>
+      <c r="C38" t="s">
+        <v>305</v>
+      </c>
+      <c r="D38" t="s">
+        <v>306</v>
+      </c>
+      <c r="E38" t="s">
+        <v>208</v>
+      </c>
+      <c r="F38" t="s">
+        <v>101</v>
+      </c>
+      <c r="G38" t="s">
+        <v>308</v>
+      </c>
+      <c r="H38">
+        <v>522</v>
+      </c>
+      <c r="I38" t="s">
+        <v>219</v>
+      </c>
+      <c r="J38" t="s">
+        <v>312</v>
+      </c>
+      <c r="K38" t="s">
+        <v>313</v>
+      </c>
+      <c r="M38" t="s">
+        <v>31</v>
+      </c>
+      <c r="N38" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -3022,12 +3152,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C9667EA7A926CE44956D0B5DCD9CC853" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d16da6adbc1ddf8797d77451e3cf87a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1d306db0-a384-4295-b85c-939a3142a74b" xmlns:ns3="a3c2bd72-a5a7-4afd-b193-b6de680f91cc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b95c06a4b98ee3d310726f4e0c3474a8" ns2:_="" ns3:_="">
     <xsd:import namespace="1d306db0-a384-4295-b85c-939a3142a74b"/>
@@ -3210,7 +3334,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3219,16 +3343,13 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3430553F-8EDA-442D-BB5A-06A762556CDB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E7D91A3-6CE8-4434-B49C-80EABACC49BC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3247,10 +3368,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB39C5E6-EEF6-4ED3-A020-8D524EF8560D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3430553F-8EDA-442D-BB5A-06A762556CDB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
20250815 - new data were added and first re-analysis
Data from EUCTR and SIRS/ACNP conferences for secondary outcomes
</commit_message>
<xml_diff>
--- a/data_u1/included_studies_2025-01-16_LSR3_H.xlsx
+++ b/data_u1/included_studies_2025-01-16_LSR3_H.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sksiafis/Documents/GitHub/LSR3_taar1_H/data_u1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC32EA9-3CAB-AB44-9EE4-278133C65F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3FE3E7-0141-3D41-B730-B9B4A6FDA84A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5300" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18880" yWindow="-22960" windowWidth="31060" windowHeight="19840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of included studies" sheetId="9" r:id="rId1"/>
@@ -301,9 +301,6 @@
     <t>NA</t>
   </si>
   <si>
-    <t xml:space="preserve">382-201-00001, NCT05593029 </t>
-  </si>
-  <si>
     <t>Sunovion/Sumitomo</t>
   </si>
   <si>
@@ -391,9 +388,6 @@
     <t>Men/women 18-55 years with schizophrenia (stable, DSM-IV-TR)</t>
   </si>
   <si>
-    <t xml:space="preserve">SEP361-108 , NCT05015673 </t>
-  </si>
-  <si>
     <t>Men/women 18-55 years with narcolepsy/cataplexy</t>
   </si>
   <si>
@@ -439,9 +433,6 @@
     <t>31.12.23</t>
   </si>
   <si>
-    <t>SEP361-124, NCT05402111 (2022)</t>
-  </si>
-  <si>
     <t>SEP361-201, NCT02969382, EUCTR2016-001555-41</t>
   </si>
   <si>
@@ -493,9 +484,6 @@
     <t>04.10.19</t>
   </si>
   <si>
-    <t>SEP361-304, NCT04115319 , EUCTR2019-002259-40</t>
-  </si>
-  <si>
     <t>SEP361-308, NCT05628103</t>
   </si>
   <si>
@@ -980,13 +968,52 @@
   </si>
   <si>
     <t>August 31 2028</t>
+  </si>
+  <si>
+    <t>SEP361-124, NCT05402111</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>382-201-00001</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, NCT05593029 </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">SEP361-108, NCT05015673 </t>
+  </si>
+  <si>
+    <r>
+      <t>SEP361-304, NCT04115319 , EUCTR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>2019-002259-40</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1007,6 +1034,18 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri (Body)"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1061,7 +1100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1099,6 +1138,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1490,7 +1530,7 @@
         <v>65</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>66</v>
@@ -1513,25 +1553,25 @@
         <v>69</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>70</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="H2" s="4">
         <v>164</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="L2">
         <v>2017</v>
@@ -1548,40 +1588,40 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="17" t="s">
         <v>73</v>
       </c>
       <c r="D3" t="s">
         <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="F3" t="s">
         <v>74</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="H3" s="9">
         <v>131</v>
       </c>
       <c r="I3" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="L3">
         <v>2023</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="N3" s="9" t="s">
         <v>77</v>
@@ -1592,7 +1632,7 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C4" t="s">
         <v>75</v>
@@ -1601,25 +1641,25 @@
         <v>69</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>76</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="H4" s="4">
         <v>287</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="L4">
         <v>2022</v>
@@ -1636,7 +1676,7 @@
         <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C5" t="s">
         <v>55</v>
@@ -1689,25 +1729,25 @@
         <v>69</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>85</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="H6" s="4">
         <v>64</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="L6">
         <v>2019</v>
@@ -1724,7 +1764,7 @@
         <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C7" t="s">
         <v>86</v>
@@ -1733,19 +1773,19 @@
         <v>69</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="H7" s="4">
         <v>49</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>86</v>
@@ -1771,31 +1811,31 @@
         <v>36</v>
       </c>
       <c r="C8" t="s">
+        <v>311</v>
+      </c>
+      <c r="D8" t="s">
         <v>87</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>89</v>
-      </c>
       <c r="G8" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="H8" s="11">
         <v>1030</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="L8" t="s">
         <v>86</v>
@@ -1809,31 +1849,31 @@
     </row>
     <row r="9" spans="1:14" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
       </c>
       <c r="C9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D9" t="s">
-        <v>88</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>92</v>
-      </c>
       <c r="G9" s="3" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="H9" s="4">
         <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>86</v>
@@ -1853,25 +1893,25 @@
     </row>
     <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B10" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E10" t="s">
         <v>78</v>
       </c>
       <c r="F10" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10" t="s">
         <v>94</v>
-      </c>
-      <c r="G10" t="s">
-        <v>95</v>
       </c>
       <c r="H10">
         <v>24</v>
@@ -1880,10 +1920,10 @@
         <v>71</v>
       </c>
       <c r="J10" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" t="s">
         <v>96</v>
-      </c>
-      <c r="K10" t="s">
-        <v>97</v>
       </c>
       <c r="L10">
         <v>2018</v>
@@ -1903,31 +1943,31 @@
         <v>27</v>
       </c>
       <c r="C11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" t="s">
+        <v>199</v>
+      </c>
+      <c r="F11" t="s">
         <v>98</v>
       </c>
-      <c r="D11" t="s">
-        <v>88</v>
-      </c>
-      <c r="E11" t="s">
-        <v>203</v>
-      </c>
-      <c r="F11" t="s">
-        <v>99</v>
-      </c>
       <c r="G11" s="5" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="H11">
         <v>13</v>
       </c>
       <c r="I11" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="L11">
         <v>2020</v>
@@ -1947,37 +1987,37 @@
         <v>30</v>
       </c>
       <c r="C12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D12" t="s">
-        <v>88</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="G12" s="3" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="H12" s="11">
         <v>83</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="L12" s="9">
         <v>2023</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="N12" t="s">
         <v>72</v>
@@ -1988,34 +2028,34 @@
         <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" t="s">
         <v>102</v>
       </c>
-      <c r="D13" t="s">
-        <v>88</v>
-      </c>
-      <c r="E13" t="s">
-        <v>103</v>
-      </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H13">
         <v>220</v>
       </c>
       <c r="I13" t="s">
+        <v>103</v>
+      </c>
+      <c r="J13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>105</v>
-      </c>
-      <c r="K13" t="s">
-        <v>106</v>
       </c>
       <c r="L13" t="s">
         <v>86</v>
@@ -2029,31 +2069,31 @@
     </row>
     <row r="14" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
         <v>56</v>
       </c>
       <c r="C14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="H14" s="4">
         <v>52</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>86</v>
@@ -2079,25 +2119,25 @@
         <v>8</v>
       </c>
       <c r="C15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" t="s">
+        <v>187</v>
+      </c>
+      <c r="F15" t="s">
         <v>109</v>
       </c>
-      <c r="D15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E15" t="s">
-        <v>191</v>
-      </c>
-      <c r="F15" t="s">
-        <v>110</v>
-      </c>
       <c r="G15" s="5" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="H15">
         <v>24</v>
       </c>
       <c r="I15" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>86</v>
@@ -2112,7 +2152,7 @@
         <v>2</v>
       </c>
       <c r="N15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2123,31 +2163,31 @@
         <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="H16" s="4">
         <v>105</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="L16">
         <v>2015</v>
@@ -2156,7 +2196,7 @@
         <v>2</v>
       </c>
       <c r="N16" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2167,31 +2207,31 @@
         <v>17</v>
       </c>
       <c r="C17" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D17" t="s">
-        <v>88</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>114</v>
-      </c>
       <c r="G17" s="3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="H17" s="4">
         <v>48</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="L17">
         <v>2014</v>
@@ -2211,31 +2251,31 @@
         <v>14</v>
       </c>
       <c r="C18" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D18" t="s">
-        <v>88</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>116</v>
-      </c>
       <c r="G18" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="H18" s="4">
         <v>48</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="L18">
         <v>2014</v>
@@ -2255,31 +2295,31 @@
         <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>117</v>
+        <v>312</v>
       </c>
       <c r="D19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="H19" s="4">
         <v>18</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="L19">
         <v>2015</v>
@@ -2288,7 +2328,7 @@
         <v>2</v>
       </c>
       <c r="N19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2299,31 +2339,31 @@
         <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="H20" s="4">
         <v>68</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="L20">
         <v>2020</v>
@@ -2332,7 +2372,7 @@
         <v>2</v>
       </c>
       <c r="N20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
@@ -2340,34 +2380,34 @@
         <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C21" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" t="s">
+        <v>119</v>
+      </c>
+      <c r="F21" t="s">
         <v>120</v>
       </c>
-      <c r="D21" t="s">
-        <v>88</v>
-      </c>
-      <c r="E21" t="s">
-        <v>121</v>
-      </c>
-      <c r="F21" t="s">
-        <v>122</v>
-      </c>
       <c r="G21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H21">
         <v>22</v>
       </c>
       <c r="I21" t="s">
+        <v>121</v>
+      </c>
+      <c r="J21" t="s">
+        <v>122</v>
+      </c>
+      <c r="K21" t="s">
         <v>123</v>
-      </c>
-      <c r="J21" t="s">
-        <v>124</v>
-      </c>
-      <c r="K21" t="s">
-        <v>125</v>
       </c>
       <c r="L21">
         <v>2023</v>
@@ -2387,31 +2427,31 @@
         <v>40</v>
       </c>
       <c r="C22" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="H22" s="4">
         <v>60</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="L22" s="14">
         <v>2024</v>
@@ -2431,31 +2471,31 @@
         <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="H23" s="16">
         <v>19</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="L23" s="14">
         <v>2024</v>
@@ -2472,34 +2512,34 @@
         <v>50</v>
       </c>
       <c r="B24" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C24" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E24" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G24" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H24">
         <v>24</v>
       </c>
       <c r="I24" t="s">
+        <v>128</v>
+      </c>
+      <c r="J24" t="s">
+        <v>129</v>
+      </c>
+      <c r="K24" t="s">
         <v>130</v>
-      </c>
-      <c r="J24" t="s">
-        <v>131</v>
-      </c>
-      <c r="K24" t="s">
-        <v>132</v>
       </c>
       <c r="L24" t="s">
         <v>86</v>
@@ -2516,34 +2556,34 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C25" t="s">
-        <v>133</v>
+        <v>310</v>
       </c>
       <c r="D25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="H25" s="11">
         <v>31</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="L25" s="9">
         <v>2023</v>
@@ -2552,7 +2592,7 @@
         <v>2</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2562,32 +2602,32 @@
       <c r="B26" t="s">
         <v>15</v>
       </c>
-      <c r="C26" t="s">
-        <v>134</v>
+      <c r="C26" s="17" t="s">
+        <v>131</v>
       </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="H26" s="4">
         <v>245</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="L26">
         <v>2018</v>
@@ -2607,31 +2647,31 @@
         <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D27" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E27" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F27" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H27">
         <v>157</v>
       </c>
       <c r="I27" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="J27" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="K27" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="L27">
         <v>2019</v>
@@ -2651,31 +2691,31 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D28" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="H28" s="4">
         <v>39</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="L28">
         <v>2023</v>
@@ -2694,32 +2734,32 @@
       <c r="B29" t="s">
         <v>38</v>
       </c>
-      <c r="C29" t="s">
-        <v>143</v>
+      <c r="C29" s="17" t="s">
+        <v>140</v>
       </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="H29" s="4">
         <v>464</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="L29" t="s">
         <v>86</v>
@@ -2738,32 +2778,32 @@
       <c r="B30" t="s">
         <v>22</v>
       </c>
-      <c r="C30" t="s">
-        <v>145</v>
+      <c r="C30" s="17" t="s">
+        <v>142</v>
       </c>
       <c r="D30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="H30" s="4">
         <v>463</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="L30">
         <v>2023</v>
@@ -2772,7 +2812,7 @@
         <v>2</v>
       </c>
       <c r="N30" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2782,32 +2822,32 @@
       <c r="B31" t="s">
         <v>24</v>
       </c>
-      <c r="C31" t="s">
-        <v>147</v>
+      <c r="C31" s="17" t="s">
+        <v>144</v>
       </c>
       <c r="D31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="H31" s="4">
         <v>462</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="L31">
         <v>2023</v>
@@ -2816,7 +2856,7 @@
         <v>2</v>
       </c>
       <c r="N31" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -2824,40 +2864,40 @@
         <v>49</v>
       </c>
       <c r="B32" t="s">
-        <v>169</v>
-      </c>
-      <c r="C32" t="s">
-        <v>148</v>
+        <v>165</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>145</v>
       </c>
       <c r="D32" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E32" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F32" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H32" s="14">
         <v>463</v>
       </c>
       <c r="I32" t="s">
+        <v>289</v>
+      </c>
+      <c r="J32" t="s">
+        <v>147</v>
+      </c>
+      <c r="K32" s="14" t="s">
         <v>293</v>
-      </c>
-      <c r="J32" t="s">
-        <v>150</v>
-      </c>
-      <c r="K32" s="14" t="s">
-        <v>297</v>
       </c>
       <c r="L32" s="14">
         <v>2023</v>
       </c>
       <c r="M32" s="14" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="N32" t="s">
         <v>72</v>
@@ -2868,34 +2908,34 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>165</v>
-      </c>
-      <c r="C33" t="s">
-        <v>151</v>
+        <v>161</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>313</v>
       </c>
       <c r="D33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="H33" s="11">
         <v>302</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="L33">
         <v>2022</v>
@@ -2912,34 +2952,34 @@
         <v>52</v>
       </c>
       <c r="B34" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C34" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D34" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E34" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F34" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G34" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H34" s="14">
         <v>101</v>
       </c>
       <c r="I34" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="J34" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="K34" s="14" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="L34" s="14">
         <v>2024</v>
@@ -2956,34 +2996,34 @@
         <v>51</v>
       </c>
       <c r="B35" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C35" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E35" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F35" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H35">
         <v>67</v>
       </c>
       <c r="I35" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="J35" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="K35" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="L35" t="s">
         <v>86</v>
@@ -2997,37 +3037,37 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B36" t="s">
-        <v>166</v>
-      </c>
-      <c r="C36" t="s">
+        <v>162</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="D36" t="s">
+        <v>87</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="G36" s="7" t="s">
         <v>273</v>
-      </c>
-      <c r="D36" t="s">
-        <v>88</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="G36" s="7" t="s">
-        <v>277</v>
       </c>
       <c r="H36" s="8">
         <v>22</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="L36">
         <v>2023</v>
@@ -3036,42 +3076,42 @@
         <v>2</v>
       </c>
       <c r="N36" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
+        <v>295</v>
+      </c>
+      <c r="B37" t="s">
+        <v>297</v>
+      </c>
+      <c r="C37" t="s">
         <v>299</v>
-      </c>
-      <c r="B37" t="s">
-        <v>301</v>
-      </c>
-      <c r="C37" t="s">
-        <v>303</v>
       </c>
       <c r="D37" t="s">
         <v>69</v>
       </c>
       <c r="E37" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="F37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G37" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="H37">
         <v>35</v>
       </c>
       <c r="I37" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="J37" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="K37" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="L37">
         <v>2019</v>
@@ -3085,37 +3125,37 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B38" t="s">
+        <v>298</v>
+      </c>
+      <c r="C38" t="s">
+        <v>301</v>
+      </c>
+      <c r="D38" t="s">
         <v>302</v>
       </c>
-      <c r="C38" t="s">
-        <v>305</v>
-      </c>
-      <c r="D38" t="s">
-        <v>306</v>
-      </c>
       <c r="E38" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G38" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="H38">
         <v>522</v>
       </c>
       <c r="I38" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J38" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="K38" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="M38" t="s">
         <v>31</v>
@@ -3152,6 +3192,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C9667EA7A926CE44956D0B5DCD9CC853" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d16da6adbc1ddf8797d77451e3cf87a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1d306db0-a384-4295-b85c-939a3142a74b" xmlns:ns3="a3c2bd72-a5a7-4afd-b193-b6de680f91cc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b95c06a4b98ee3d310726f4e0c3474a8" ns2:_="" ns3:_="">
     <xsd:import namespace="1d306db0-a384-4295-b85c-939a3142a74b"/>
@@ -3334,22 +3389,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3430553F-8EDA-442D-BB5A-06A762556CDB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB39C5E6-EEF6-4ED3-A020-8D524EF8560D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E7D91A3-6CE8-4434-B49C-80EABACC49BC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3366,21 +3423,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB39C5E6-EEF6-4ED3-A020-8D524EF8560D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3430553F-8EDA-442D-BB5A-06A762556CDB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>